<commit_message>
Avance de PDF de OC
</commit_message>
<xml_diff>
--- a/src/main/java/com/mycompany/ocxrst/BASES/INVENTARIOS.xlsx
+++ b/src/main/java/com/mycompany/ocxrst/BASES/INVENTARIOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OCXRST\OrdendeComprasRST\src\main\java\com\mycompany\ocxrst\BASES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9937B966-F8E3-4C79-8906-B9F33905FA5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{156E3ABC-3A4B-41D7-B90B-DA0F5805BFDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4800" yWindow="2980" windowWidth="14400" windowHeight="8170" xr2:uid="{07BBAD01-711C-41B6-957E-FFFDE243DC03}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{07BBAD01-711C-41B6-957E-FFFDE243DC03}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>